<commit_message>
Test plan: add g02-g17 12 Oct traffic validation + TC-CTL-036 results
TC-AFM-002/003/004, L1 TC-AFM-005 (RCCL cross-domain), TC-HW-008 PASS from the
18-tray TransferBench/RCCL smoke validation; TC-CTL-036 PASS from the 10 Oct
post-bringup gate; TC-AFM-001 note only (sysfs, no L2 ping).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testplan/HPE_AMD Helios Juniper ScaleUp TestPlan.xlsx
+++ b/testplan/HPE_AMD Helios Juniper ScaleUp TestPlan.xlsx
@@ -5080,7 +5080,7 @@
       </c>
       <c r="H2" s="23" t="inlineStr">
         <is>
-          <t>Execution Notes (g02-g17 full rack (6 sw / 17 CT), 10-11 Oct 2026)</t>
+          <t>Execution Notes (g02-g17 full rack (6 sw / 17-18 CT), 10-12 Oct 2026)</t>
         </is>
       </c>
     </row>
@@ -5105,6 +5105,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H3" s="27" t="inlineStr">
+        <is>
+          <t>Partial evidence (12 Oct, S8 UALink sysfs): 72/72 accelerators active, vpod_id=1 and correct local_accels on all 18 trays. afmctl L2 ping was not part of that run, so status not set.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -5127,6 +5132,21 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>RACK-BKC-RCRD-26.12-rc5; AFM 0.1.0-AIFM-817</t>
+        </is>
+      </c>
+      <c r="H4" s="27" t="inlineStr">
+        <is>
+          <t>12 Oct traffic validation T1: TransferBench v1.70.02 (b82b036) smoketest on every tray, 4 GPUs each; PASS 18/18 trays ('All tests passed', exit 0).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -5149,6 +5169,21 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>RACK-BKC-RCRD-26.12-rc5; AFM 0.1.0-AIFM-817</t>
+        </is>
+      </c>
+      <c r="H5" s="27" t="inlineStr">
+        <is>
+          <t>12 Oct traffic validation T2: LaunchTransferBench.sh smoketest from CT01 across 18 trays / 72 GPUs (18 ranks, H2D/D2H/D2D remote write+read); all transfers passed, exit 0.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -5171,6 +5206,21 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>RACK-BKC-RCRD-26.12-rc5; AFM 0.1.0-AIFM-817</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>12 Oct traffic validation T3: RcclSmokeTest v1.0.0 (d03571d), 7 collectives x 1 KB/4 MB/1 GB per tray; PASS 18/18 trays (21/21 cells each). Needs NCCL_IB_DISABLE=1 NCCL_CUMEM_ENABLE=0.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -5191,6 +5241,21 @@
       <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>RACK-BKC-RCRD-26.12-rc5; AFM 0.1.0-AIFM-817</t>
+        </is>
+      </c>
+      <c r="H7" s="27" t="inlineStr">
+        <is>
+          <t>12 Oct traffic validation T4: RcclSmokeTest across 18 trays / 72 ranks from CT01; 21/21 cells incl. 1 GB, all processes exited cleanly, exit 0.</t>
         </is>
       </c>
     </row>
@@ -10109,6 +10174,21 @@
           <t>Cluster and all quorum nodes is healthy</t>
         </is>
       </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>AFM 0.1.0-AICC-817</t>
+        </is>
+      </c>
+      <c r="H233" s="27" t="inlineStr">
+        <is>
+          <t>10 Oct post-bringup gate: cluster healthy=true, leader 10.190.198.49, 3/3 quorum members (.49/.50/.51) started with conditions true.</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="9" t="inlineStr">
@@ -11559,6 +11639,21 @@
       <c r="D314" t="inlineStr">
         <is>
           <t>Inprogress</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>RACK-BKC-RCRD-26.12-rc5; AFM 0.1.0-AIFM-817</t>
+        </is>
+      </c>
+      <c r="H314" s="27" t="inlineStr">
+        <is>
+          <t>Covered by 12 Oct traffic validation T1: TransferBench smoketest (includes All-to-All remote write/read) in-domain on all 18 trays, PASS 18/18.</t>
         </is>
       </c>
     </row>
@@ -16060,6 +16155,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="31" t="inlineStr">
         <is>
@@ -16171,6 +16267,8 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="34" t="inlineStr">
         <is>
@@ -16181,14 +16279,14 @@
     <row r="16">
       <c r="A16" s="35" t="inlineStr">
         <is>
-          <t>Rack: g02-g17 full rack (6 sw / 17 CT), 10-11 Oct 2026. Switches 10.190.198.46-.51 (controllers .51/.50/.49), 17 compute trays x 4 GPUs (68 GPUs), sideband control mode, not MCH.</t>
+          <t>Rack: g02-g17 full rack (6 sw / 17 CT), 10-11 Oct 2026 (AFM L2 batch); 12 Oct 2026 traffic validation with all 18 compute trays (72 GPUs) admitted. Switches 10.190.198.46-.51 (controllers .51/.50/.49), 17 compute trays x 4 GPUs (68 GPUs), sideband control mode, not MCH.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="35" t="inlineStr">
         <is>
-          <t>Software: AFM 0.1.0-AICC-817 (vcs 7f4afe07a, built 2026-10-05); ROCm 10.2.0; RCCL 2.31.2; amdgpu 3.65.0; afmctl 0.0.1-85.</t>
+          <t>Software: AFM 0.1.0-AICC-817 (vcs 7f4afe07a, built 2026-10-05); ROCm 10.2.0; RCCL 2.31.2; amdgpu 3.65.0; afmctl 0.0.1-85. 12 Oct traffic validation: RACK-BKC-RCRD-26.12-rc5, ROCm 10.2.0a20260922, amdgpu 7.1.0, IFoE 0.2.10.1000, afmctl 0.0.1-94, TransferBench v1.70.02, RcclSmokeTest v1.0.0, SONiC 202505I20260915.</t>
         </is>
       </c>
     </row>
@@ -16216,7 +16314,7 @@
     <row r="21">
       <c r="A21" s="35" t="inlineStr">
         <is>
-          <t>Source: results/full_rack-command-log.md (contains plaintext credentials - do not share unredacted).</t>
+          <t>Source: results/AMD-Fullrack-logs/command-log.md (10-11 Oct; contains plaintext credentials - do not share unredacted) and g02-g17-traffic-validation-20261012.md (12 Oct).</t>
         </is>
       </c>
     </row>

</xml_diff>